<commit_message>
resolved extent report bug
</commit_message>
<xml_diff>
--- a/excel_test_output/TestCasesStatus.xlsx
+++ b/excel_test_output/TestCasesStatus.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="31">
   <si>
     <t>S_No.</t>
   </si>
@@ -23,12 +23,57 @@
     <t>STATUS</t>
   </si>
   <si>
+    <t>testWithoutSelectingAnyMember</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>testCoupleChildrenAgeGapLess18</t>
+  </si>
+  <si>
+    <t>testWithoutPinCode</t>
+  </si>
+  <si>
+    <t>testEditMemberDetailsButton</t>
+  </si>
+  <si>
+    <t>testHealthInsurance</t>
+  </si>
+  <si>
+    <t>validateContactUsPage</t>
+  </si>
+  <si>
+    <t>invalidPhoneNumberTest</t>
+  </si>
+  <si>
+    <t>missingPolicyIdTest</t>
+  </si>
+  <si>
+    <t>successfulSubmissionTest</t>
+  </si>
+  <si>
+    <t>invalidEmailTest</t>
+  </si>
+  <si>
+    <t>testNavigateToCarInsurance</t>
+  </si>
+  <si>
+    <t>testEnterPincodeAndProceed</t>
+  </si>
+  <si>
+    <t>testSelectCarDetails</t>
+  </si>
+  <si>
+    <t>testReviewAndProceed</t>
+  </si>
+  <si>
+    <t>testVerifyPlansAndDetails</t>
+  </si>
+  <si>
     <t>testNavigationToBikeSection</t>
   </si>
   <si>
-    <t>PASS</t>
-  </si>
-  <si>
     <t>testRegistrationErrorValidation</t>
   </si>
   <si>
@@ -44,10 +89,13 @@
     <t>testWorkmenCompensationOpensInNewTab</t>
   </si>
   <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>testSubmitWithoutDetails</t>
+  </si>
+  <si>
     <t>SKIP</t>
-  </si>
-  <si>
-    <t>testSubmitWithoutDetails</t>
   </si>
   <si>
     <t>testValidDetailsSubmission</t>
@@ -73,7 +121,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -86,6 +134,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="17"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="10"/>
       </patternFill>
     </fill>
     <fill>
@@ -106,25 +159,40 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -201,7 +269,7 @@
         <v>9</v>
       </c>
       <c r="C7" t="s" s="6">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -209,10 +277,10 @@
         <v>7.0</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s" s="7">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -220,10 +288,10 @@
         <v>8.0</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s" s="8">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -231,10 +299,10 @@
         <v>9.0</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s" s="9">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -242,10 +310,175 @@
         <v>10.0</v>
       </c>
       <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s" s="10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11.0</v>
+      </c>
+      <c r="B12" t="s">
         <v>14</v>
       </c>
-      <c r="C11" t="s" s="10">
-        <v>10</v>
+      <c r="C12" t="s" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12.0</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13.0</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" t="s" s="13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14.0</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s" s="14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15.0</v>
+      </c>
+      <c r="B16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" t="s" s="15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16.0</v>
+      </c>
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" t="s" s="16">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17.0</v>
+      </c>
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" t="s" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18.0</v>
+      </c>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" t="s" s="18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19.0</v>
+      </c>
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" t="s" s="19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="B21" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" t="s" s="20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21.0</v>
+      </c>
+      <c r="B22" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" t="s" s="21">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22.0</v>
+      </c>
+      <c r="B23" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" t="s" s="22">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23.0</v>
+      </c>
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s" s="23">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24.0</v>
+      </c>
+      <c r="B25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" t="s" s="24">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25.0</v>
+      </c>
+      <c r="B26" t="s">
+        <v>30</v>
+      </c>
+      <c r="C26" t="s" s="25">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>